<commit_message>
Work in progress - Dec 22, 2025 before shutdown
- Modified MAIN_1_CoAnQi.cpp (5.51 MB, last worked Dec 10)
- Updated CMakeLists.txt
- Updated .gitignore
- Removed MP4 video files from inbox-dropzone
- Added safety backups and checkpoint documentation

Preserving state before VS Code shutdown.
</commit_message>
<xml_diff>
--- a/inbox-dropzone/Grok_clone access_backup.xlsx
+++ b/inbox-dropzone/Grok_clone access_backup.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="30" windowWidth="18855" windowHeight="7185" firstSheet="7" activeTab="10"/>
+    <workbookView xWindow="240" yWindow="30" windowWidth="18855" windowHeight="7185" firstSheet="9" activeTab="11"/>
   </bookViews>
   <sheets>
     <sheet name="Clone" sheetId="1" r:id="rId1"/>
@@ -18,13 +18,14 @@
     <sheet name="Discoveries" sheetId="9" r:id="rId9"/>
     <sheet name="Source4 full integration plan" sheetId="10" r:id="rId10"/>
     <sheet name="06Workspace Cleanup" sheetId="11" r:id="rId11"/>
+    <sheet name="Hoja4" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3404" uniqueCount="3158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3478" uniqueCount="3231">
   <si>
     <t>https://github.com/Daniel8Murphy0007/Star-Magic</t>
   </si>
@@ -18192,6 +18193,480 @@
         <family val="2"/>
       </rPr>
       <t> on clean workspace</t>
+    </r>
+  </si>
+  <si>
+    <t>Proceed with suggestions before phase 1 integration:1. Create comprehensive .gitignore; 2. Clean log files and build artifacts; 3. Verify git status shows &lt;50 files; 4. Test git add . on clean workspace</t>
+  </si>
+  <si>
+    <t>The WORKSPACE_BACKUP_739PM directory contains files exceeding GitHub's 100 MB limit. We need to exclude it from git:</t>
+  </si>
+  <si>
+    <t>Successfully removed from git tracking. Now let's amend the commit to finalize the cleanup:</t>
+  </si>
+  <si>
+    <t>Excellent! Push successful. Now verify the current state:</t>
+  </si>
+  <si>
+    <t>Perfect! Git is clean (only 1 modified file - likely .gitignore locally). Now we can proceed with Phase 1 integration. Let me start by reading the source files to extract the 46 PhysicsTerm classes:</t>
+  </si>
+  <si>
+    <t>I can see the source files clearly. Now I'll proceed with Phase 1 integration systematically. Let me read the complete class definitions from all three files and then integrate them into MAIN_1_CoAnQi.cpp. Given the large amount of code to integrate (~1,700 lines), I'll do this in organized batches.</t>
+  </si>
+  <si>
+    <t>First, let me check the insertion point in MAIN_1_CoAnQi.cpp:</t>
+  </si>
+  <si>
+    <t>Given the scope of this integration (~1,700 lines), let me create a comprehensive implementation plan and execute it systematically. Due to the conversation approaching token limits, I'll provide you with a detailed status update showing what needs to be done:</t>
+  </si>
+  <si>
+    <t>Phase 1 Integration Status</t>
+  </si>
+  <si>
+    <t>COMPLETED:</t>
+  </si>
+  <si>
+    <t>✅ Workspace cleanup (113 logs + backups removed)</t>
+  </si>
+  <si>
+    <t>✅ .gitignore enhanced (25+ patterns including WORKSPACE_BACKUP_*/)</t>
+  </si>
+  <si>
+    <t>✅ Git push successful (commit 2079b6a)</t>
+  </si>
+  <si>
+    <t>✅ PhysicsTerm base class conflict resolved (using ::PhysicsTerm; at line 25841)</t>
+  </si>
+  <si>
+    <t>✅ Workspace ready (git status clean)</t>
+  </si>
+  <si>
+    <t>IMMEDIATE NEXT STEP - Phase 1 Integration:</t>
+  </si>
+  <si>
+    <t>Files to extract from:</t>
+  </si>
+  <si>
+    <t>1. source4_wolfram.cpp (24 classes, 870 lines)</t>
+  </si>
+  <si>
+    <t>2. source4_wolfram_compressed.cpp (9 classes, 312 lines)</t>
+  </si>
+  <si>
+    <t>3. source4_wolfram_resonance.cpp (13 classes, 628 lines)</t>
+  </si>
+  <si>
+    <t>Integration approach:</t>
+  </si>
+  <si>
+    <t>Due to the size (~1,700 lines), would you like me to:</t>
+  </si>
+  <si>
+    <t>1. First commit: 8 UQFF core classes (~200 lines)</t>
+  </si>
+  <si>
+    <t>2. Second commit: 6 helper classes (~150 lines)</t>
+  </si>
+  <si>
+    <t>3. Third commit: 9 MUGE compressed + 13 MUGE resonance (~700 lines)</t>
+  </si>
+  <si>
+    <t>4. Fourth commit: 7 system classes + 3 misc (~400 lines)</t>
+  </si>
+  <si>
+    <t>5. Fifth commit: FluidSolver class (~600 lines)</t>
+  </si>
+  <si>
+    <t>6. Sixth commit: DualMethodValidator (~400 lines)</t>
+  </si>
+  <si>
+    <r>
+      <t>Perfect! I can see the namespace SOURCE4 ends at line 26233 and SOURCE82 integration starts at line 26235. I need to insert the 46 PhysicsTerm classes just before line 26233 (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>} // namespace SOURCE4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>I've confirmed the files and insertion point. The 46 PhysicsTerm classes need to be inserted starting at line ~26027 (after SOURCE4 inline functions, before </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>} // namespace SOURCE4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> at line 26233).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Option A:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> Complete the full Phase 1 integration in one comprehensive edit (all 46 classes + FluidSolver + DualMethodValidator ~2,700 lines total)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Option B:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> Break into smaller commits:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Option C:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> Save current session documentation and start fresh with Phase 1 execution in new conversation</t>
+    </r>
+  </si>
+  <si>
+    <t>Option C, proceed</t>
+  </si>
+  <si>
+    <t>Excellent! ✅ Session saved successfully. Final summary:</t>
+  </si>
+  <si>
+    <t>Session Complete - Ready for Phase 1</t>
+  </si>
+  <si>
+    <t>Git Status:</t>
+  </si>
+  <si>
+    <t>Commit 84d34d6 pushed to origin/master</t>
+  </si>
+  <si>
+    <t>Workspace clean and ready</t>
+  </si>
+  <si>
+    <t>All documentation saved</t>
+  </si>
+  <si>
+    <t>Documentation Created:</t>
+  </si>
+  <si>
+    <t>1. COPILOT_SESSION_SOURCE4_PHASE1_Dec6_2025_0930AM.md (707 lines) - Detailed integration plan</t>
+  </si>
+  <si>
+    <t>2. COPILOT_SESSION_CLEANUP_COMPLETE_Dec7_2025.md (655 lines) - This session summary</t>
+  </si>
+  <si>
+    <t>Next Session Prompt:</t>
+  </si>
+  <si>
+    <t>Continue with SOURCE4 Phase 1 integration: Integrate 46 PhysicsTerm classes + FluidSolver + DualMethodValidator into MAIN_1_CoAnQi.cpp namespace SOURCE4.</t>
+  </si>
+  <si>
+    <t>See COPILOT_SESSION_CLEANUP_COMPLETE_Dec7_2025.md for complete context and action items.</t>
+  </si>
+  <si>
+    <t>PERFECT! THE WORK IS COMPLETE AND ALREADY IN THE INDEX!</t>
+  </si>
+  <si>
+    <t>PROOF:</t>
+  </si>
+  <si>
+    <t>CURRENT STATUS:</t>
+  </si>
+  <si>
+    <t>The 37 PhysicsTerm classes ARE ALREADY INTEGRATED into MAIN_1_CoAnQi.cpp!</t>
+  </si>
+  <si>
+    <t>WHAT'S INTEGRATED (Lines 26234-26956):</t>
+  </si>
+  <si>
+    <t>6 Helper classes ✅</t>
+  </si>
+  <si>
+    <t>6 UQFF classes ✅</t>
+  </si>
+  <si>
+    <t>7 MUGE Compressed classes ✅</t>
+  </si>
+  <si>
+    <t>13 MUGE Resonance classes ✅</t>
+  </si>
+  <si>
+    <t>WHAT'S STILL MISSING:</t>
+  </si>
+  <si>
+    <t>5 missing classes from partial integration</t>
+  </si>
+  <si>
+    <t>7 System classes</t>
+  </si>
+  <si>
+    <t>3 Misc classes</t>
+  </si>
+  <si>
+    <t>FluidSolver</t>
+  </si>
+  <si>
+    <t>DualMethodValidator</t>
+  </si>
+  <si>
+    <t>DO YOU WANT TO:</t>
+  </si>
+  <si>
+    <r>
+      <t>✅ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>Git index SHA:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>4d0603c76e43e1c1210a86f51f8191a4a4f846f4</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>✅ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>Working file SHA:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>4d0603c76e43e1c1210a86f51f8191a4a4f846f4</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>✅ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>THEY MATCH!</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> File is already staged/indexed!</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>✅ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>File ends at line 105,577</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> with proper closure</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>✅ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>Last commit has 93,164 lines</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> (the old version)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>✅ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>Difference:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> +12,413 lines added (the 37 PhysicsTerm classes!)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>They're just </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>waiting to be committed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>. The work was completed during the interrupted session and the file is sitting in the git index, ready to commit.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>TOTAL: 32 classes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> (not 37)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1. COMMIT what's already done</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> (32 classes, +12,413 lines)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2. ADD the remaining components</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> BEFORE committing</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>3. REVIEW what's there</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> line by line first</t>
     </r>
   </si>
 </sst>
@@ -18199,7 +18674,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -18368,6 +18843,11 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="15"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -18510,7 +18990,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="219">
+  <cellXfs count="224">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
@@ -18998,9 +19478,6 @@
     <xf numFmtId="0" fontId="20" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="2"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -19015,6 +19492,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -19078,11 +19559,21 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="3"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -19524,7 +20015,7 @@
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" t="s">
+      <c r="A5" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B5" t="s">
@@ -19548,6 +20039,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A5" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -19698,27 +20192,27 @@
       <c r="D38" s="32"/>
     </row>
     <row r="39" spans="4:4">
-      <c r="D39" s="216" t="s">
+      <c r="D39" s="217" t="s">
         <v>2826</v>
       </c>
     </row>
     <row r="40" spans="4:4">
-      <c r="D40" s="216" t="s">
+      <c r="D40" s="217" t="s">
         <v>2827</v>
       </c>
     </row>
     <row r="41" spans="4:4">
-      <c r="D41" s="216" t="s">
+      <c r="D41" s="217" t="s">
         <v>2828</v>
       </c>
     </row>
     <row r="42" spans="4:4">
-      <c r="D42" s="216" t="s">
+      <c r="D42" s="217" t="s">
         <v>2829</v>
       </c>
     </row>
     <row r="43" spans="4:4">
-      <c r="D43" s="216" t="s">
+      <c r="D43" s="217" t="s">
         <v>2830</v>
       </c>
     </row>
@@ -19731,7 +20225,7 @@
       <c r="D45" s="32"/>
     </row>
     <row r="46" spans="4:4" ht="28.5">
-      <c r="D46" s="216" t="s">
+      <c r="D46" s="217" t="s">
         <v>2832</v>
       </c>
     </row>
@@ -19744,7 +20238,7 @@
       <c r="D48" s="32"/>
     </row>
     <row r="49" spans="4:4">
-      <c r="D49" s="216" t="s">
+      <c r="D49" s="217" t="s">
         <v>2834</v>
       </c>
     </row>
@@ -21019,261 +21513,261 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="C5:D180"/>
+  <dimension ref="C5:D247"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="4" max="4" width="91.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="5" spans="4:4" ht="28.5">
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="95" t="s">
         <v>3025</v>
       </c>
     </row>
     <row r="6" spans="4:4" ht="28.5">
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="106" t="s">
         <v>3050</v>
       </c>
     </row>
     <row r="7" spans="4:4">
-      <c r="D7" s="217"/>
+      <c r="D7" s="218"/>
     </row>
     <row r="8" spans="4:4" ht="30">
-      <c r="D8" s="23" t="s">
+      <c r="D8" s="111" t="s">
         <v>3026</v>
       </c>
     </row>
     <row r="9" spans="4:4">
-      <c r="D9" s="187" t="s">
+      <c r="D9" s="120" t="s">
         <v>3051</v>
       </c>
     </row>
     <row r="10" spans="4:4" ht="28.5">
-      <c r="D10" s="187" t="s">
+      <c r="D10" s="120" t="s">
         <v>3052</v>
       </c>
     </row>
     <row r="11" spans="4:4">
-      <c r="D11" s="43"/>
+      <c r="D11" s="194"/>
     </row>
     <row r="12" spans="4:4">
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="95" t="s">
         <v>3027</v>
       </c>
     </row>
     <row r="13" spans="4:4">
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="95" t="s">
         <v>3053</v>
       </c>
     </row>
     <row r="14" spans="4:4">
-      <c r="D14" s="217"/>
+      <c r="D14" s="218"/>
     </row>
     <row r="15" spans="4:4">
-      <c r="D15" s="32" t="s">
+      <c r="D15" s="110" t="s">
         <v>3028</v>
       </c>
     </row>
     <row r="16" spans="4:4">
-      <c r="D16" s="32" t="s">
+      <c r="D16" s="110" t="s">
         <v>3029</v>
       </c>
     </row>
     <row r="17" spans="4:4">
-      <c r="D17" s="32" t="s">
+      <c r="D17" s="110" t="s">
         <v>3030</v>
       </c>
     </row>
     <row r="18" spans="4:4">
-      <c r="D18" s="23" t="s">
+      <c r="D18" s="111" t="s">
         <v>3031</v>
       </c>
     </row>
     <row r="19" spans="4:4">
-      <c r="D19" s="43"/>
+      <c r="D19" s="194"/>
     </row>
     <row r="20" spans="4:4">
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="95" t="s">
         <v>3054</v>
       </c>
     </row>
     <row r="21" spans="4:4">
-      <c r="D21" s="217"/>
+      <c r="D21" s="218"/>
     </row>
     <row r="22" spans="4:4">
-      <c r="D22" s="32" t="s">
+      <c r="D22" s="110" t="s">
         <v>3032</v>
       </c>
     </row>
     <row r="23" spans="4:4">
-      <c r="D23" s="32" t="s">
+      <c r="D23" s="110" t="s">
         <v>3033</v>
       </c>
     </row>
     <row r="24" spans="4:4">
-      <c r="D24" s="32" t="s">
+      <c r="D24" s="110" t="s">
         <v>3034</v>
       </c>
     </row>
     <row r="25" spans="4:4">
-      <c r="D25" s="43"/>
+      <c r="D25" s="194"/>
     </row>
     <row r="26" spans="4:4" ht="28.5">
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="106" t="s">
         <v>3055</v>
       </c>
     </row>
     <row r="27" spans="4:4">
-      <c r="D27" s="217"/>
+      <c r="D27" s="218"/>
     </row>
     <row r="28" spans="4:4">
-      <c r="D28" s="32" t="s">
+      <c r="D28" s="110" t="s">
         <v>3035</v>
       </c>
     </row>
     <row r="29" spans="4:4">
-      <c r="D29" s="32" t="s">
+      <c r="D29" s="110" t="s">
         <v>3056</v>
       </c>
     </row>
     <row r="30" spans="4:4">
-      <c r="D30" s="23" t="s">
+      <c r="D30" s="111" t="s">
         <v>3036</v>
       </c>
     </row>
     <row r="31" spans="4:4">
-      <c r="D31" s="43"/>
+      <c r="D31" s="194"/>
     </row>
     <row r="32" spans="4:4">
-      <c r="D32" s="8" t="s">
+      <c r="D32" s="95" t="s">
         <v>3037</v>
       </c>
     </row>
     <row r="33" spans="4:4">
-      <c r="D33" s="7" t="s">
+      <c r="D33" s="106" t="s">
         <v>3057</v>
       </c>
     </row>
     <row r="34" spans="4:4" ht="28.5">
-      <c r="D34" s="7" t="s">
+      <c r="D34" s="106" t="s">
         <v>3058</v>
       </c>
     </row>
     <row r="35" spans="4:4">
-      <c r="D35" s="43"/>
+      <c r="D35" s="194"/>
     </row>
     <row r="36" spans="4:4">
-      <c r="D36" s="8" t="s">
+      <c r="D36" s="95" t="s">
         <v>3038</v>
       </c>
     </row>
     <row r="37" spans="4:4" ht="28.5">
-      <c r="D37" s="21" t="s">
+      <c r="D37" s="109" t="s">
         <v>3039</v>
       </c>
     </row>
     <row r="38" spans="4:4" ht="17.25">
-      <c r="D38" s="185" t="s">
+      <c r="D38" s="190" t="s">
         <v>3040</v>
       </c>
     </row>
     <row r="39" spans="4:4">
-      <c r="D39" s="7" t="s">
+      <c r="D39" s="106" t="s">
         <v>3041</v>
       </c>
     </row>
     <row r="40" spans="4:4">
-      <c r="D40" s="7" t="s">
+      <c r="D40" s="106" t="s">
         <v>3059</v>
       </c>
     </row>
     <row r="41" spans="4:4">
-      <c r="D41" s="217"/>
+      <c r="D41" s="218"/>
     </row>
     <row r="42" spans="4:4">
-      <c r="D42" s="187" t="s">
+      <c r="D42" s="120" t="s">
         <v>3060</v>
       </c>
     </row>
     <row r="43" spans="4:4">
-      <c r="D43" s="32"/>
+      <c r="D43" s="110"/>
     </row>
     <row r="44" spans="4:4">
-      <c r="D44" s="218" t="s">
+      <c r="D44" s="219" t="s">
         <v>3042</v>
       </c>
     </row>
     <row r="45" spans="4:4">
-      <c r="D45" s="216" t="s">
+      <c r="D45" s="220" t="s">
         <v>3061</v>
       </c>
     </row>
     <row r="46" spans="4:4">
-      <c r="D46" s="216" t="s">
+      <c r="D46" s="220" t="s">
         <v>3043</v>
       </c>
     </row>
     <row r="47" spans="4:4">
-      <c r="D47" s="216" t="s">
+      <c r="D47" s="220" t="s">
         <v>3044</v>
       </c>
     </row>
     <row r="48" spans="4:4">
-      <c r="D48" s="187" t="s">
+      <c r="D48" s="120" t="s">
         <v>3062</v>
       </c>
     </row>
     <row r="49" spans="3:4">
-      <c r="D49" s="32"/>
+      <c r="D49" s="110"/>
     </row>
     <row r="50" spans="3:4">
-      <c r="D50" s="216" t="s">
+      <c r="D50" s="220" t="s">
         <v>3063</v>
       </c>
     </row>
     <row r="51" spans="3:4">
-      <c r="D51" s="216" t="s">
+      <c r="D51" s="220" t="s">
         <v>3045</v>
       </c>
     </row>
     <row r="52" spans="3:4">
-      <c r="D52" s="216" t="s">
+      <c r="D52" s="220" t="s">
         <v>3046</v>
       </c>
     </row>
     <row r="53" spans="3:4">
-      <c r="D53" s="187" t="s">
+      <c r="D53" s="120" t="s">
         <v>3064</v>
       </c>
     </row>
     <row r="54" spans="3:4">
-      <c r="D54" s="32"/>
+      <c r="D54" s="110"/>
     </row>
     <row r="55" spans="3:4">
-      <c r="D55" s="218" t="s">
+      <c r="D55" s="219" t="s">
         <v>3047</v>
       </c>
     </row>
     <row r="56" spans="3:4">
-      <c r="D56" s="216" t="s">
+      <c r="D56" s="220" t="s">
         <v>3065</v>
       </c>
     </row>
     <row r="57" spans="3:4">
-      <c r="D57" s="218" t="s">
+      <c r="D57" s="219" t="s">
         <v>3048</v>
       </c>
     </row>
     <row r="58" spans="3:4">
-      <c r="D58" s="43"/>
+      <c r="D58" s="194"/>
     </row>
     <row r="59" spans="3:4">
-      <c r="D59" s="7" t="s">
+      <c r="D59" s="106" t="s">
         <v>3049</v>
       </c>
     </row>
     <row r="60" spans="3:4">
-      <c r="D60" t="s">
+      <c r="D60" s="193" t="s">
         <v>3067</v>
       </c>
     </row>
@@ -21281,500 +21775,810 @@
       <c r="C61" t="s">
         <v>3068</v>
       </c>
-      <c r="D61" t="s">
+      <c r="D61" s="193" t="s">
         <v>3066</v>
       </c>
     </row>
+    <row r="62" spans="3:4">
+      <c r="D62" s="193"/>
+    </row>
     <row r="63" spans="3:4">
-      <c r="D63" s="8" t="s">
+      <c r="D63" s="95" t="s">
         <v>3069</v>
       </c>
     </row>
     <row r="64" spans="3:4">
-      <c r="D64" s="20"/>
+      <c r="D64" s="107"/>
     </row>
     <row r="65" spans="4:4">
-      <c r="D65" s="21" t="s">
+      <c r="D65" s="109" t="s">
         <v>3070</v>
       </c>
     </row>
     <row r="66" spans="4:4">
-      <c r="D66" s="21" t="s">
+      <c r="D66" s="109" t="s">
         <v>3071</v>
       </c>
     </row>
     <row r="67" spans="4:4">
-      <c r="D67" s="21" t="s">
+      <c r="D67" s="109" t="s">
         <v>3072</v>
       </c>
     </row>
     <row r="68" spans="4:4">
-      <c r="D68" s="5"/>
+      <c r="D68" s="97"/>
     </row>
     <row r="69" spans="4:4">
-      <c r="D69" s="7" t="s">
+      <c r="D69" s="106" t="s">
         <v>3073</v>
       </c>
     </row>
     <row r="70" spans="4:4">
-      <c r="D70" s="8" t="s">
+      <c r="D70" s="95" t="s">
         <v>3074</v>
       </c>
     </row>
     <row r="71" spans="4:4">
-      <c r="D71" s="20"/>
+      <c r="D71" s="107"/>
     </row>
     <row r="72" spans="4:4">
-      <c r="D72" s="22" t="s">
+      <c r="D72" s="113" t="s">
         <v>3081</v>
       </c>
     </row>
     <row r="73" spans="4:4">
-      <c r="D73" s="22" t="s">
+      <c r="D73" s="113" t="s">
         <v>3082</v>
       </c>
     </row>
     <row r="74" spans="4:4">
-      <c r="D74" s="24" t="s">
+      <c r="D74" s="119" t="s">
         <v>3083</v>
       </c>
     </row>
     <row r="75" spans="4:4">
-      <c r="D75" s="23" t="s">
+      <c r="D75" s="111" t="s">
         <v>3075</v>
       </c>
     </row>
     <row r="76" spans="4:4">
-      <c r="D76" s="23" t="s">
+      <c r="D76" s="111" t="s">
         <v>3076</v>
       </c>
     </row>
     <row r="77" spans="4:4">
-      <c r="D77" s="23" t="s">
+      <c r="D77" s="111" t="s">
         <v>3077</v>
       </c>
     </row>
     <row r="78" spans="4:4">
-      <c r="D78" s="22" t="s">
+      <c r="D78" s="113" t="s">
         <v>3084</v>
       </c>
     </row>
     <row r="79" spans="4:4">
-      <c r="D79" s="23" t="s">
+      <c r="D79" s="111" t="s">
         <v>3078</v>
       </c>
     </row>
     <row r="80" spans="4:4">
-      <c r="D80" s="23" t="s">
+      <c r="D80" s="111" t="s">
         <v>1835</v>
       </c>
     </row>
     <row r="81" spans="4:4">
-      <c r="D81" s="32" t="s">
+      <c r="D81" s="110" t="s">
         <v>3085</v>
       </c>
     </row>
     <row r="82" spans="4:4">
-      <c r="D82" s="5"/>
+      <c r="D82" s="97"/>
     </row>
     <row r="83" spans="4:4">
-      <c r="D83" s="7" t="s">
+      <c r="D83" s="106" t="s">
         <v>3079</v>
       </c>
     </row>
     <row r="84" spans="4:4">
-      <c r="D84" s="5"/>
+      <c r="D84" s="97"/>
     </row>
     <row r="85" spans="4:4">
-      <c r="D85" s="7" t="s">
+      <c r="D85" s="106" t="s">
         <v>3080</v>
       </c>
     </row>
+    <row r="86" spans="4:4">
+      <c r="D86" s="193"/>
+    </row>
     <row r="87" spans="4:4">
-      <c r="D87" t="s">
+      <c r="D87" s="193" t="s">
         <v>3086</v>
       </c>
     </row>
     <row r="88" spans="4:4">
-      <c r="D88" t="s">
+      <c r="D88" s="193" t="s">
         <v>3087</v>
       </c>
     </row>
     <row r="89" spans="4:4">
-      <c r="D89" t="s">
+      <c r="D89" s="193" t="s">
         <v>3088</v>
       </c>
     </row>
     <row r="90" spans="4:4">
-      <c r="D90" t="s">
+      <c r="D90" s="193" t="s">
         <v>3089</v>
       </c>
     </row>
+    <row r="91" spans="4:4">
+      <c r="D91" s="193"/>
+    </row>
     <row r="92" spans="4:4">
-      <c r="D92" t="s">
+      <c r="D92" s="193" t="s">
         <v>3090</v>
       </c>
     </row>
     <row r="93" spans="4:4">
-      <c r="D93" t="s">
+      <c r="D93" s="193" t="s">
         <v>3091</v>
       </c>
     </row>
     <row r="94" spans="4:4">
-      <c r="D94" t="s">
+      <c r="D94" s="193" t="s">
         <v>3092</v>
       </c>
     </row>
     <row r="95" spans="4:4">
-      <c r="D95" t="s">
+      <c r="D95" s="193" t="s">
         <v>3093</v>
       </c>
     </row>
     <row r="96" spans="4:4">
-      <c r="D96" t="s">
+      <c r="D96" s="193" t="s">
         <v>3094</v>
       </c>
     </row>
     <row r="97" spans="4:4">
-      <c r="D97" t="s">
+      <c r="D97" s="193" t="s">
         <v>3095</v>
       </c>
     </row>
     <row r="98" spans="4:4">
-      <c r="D98" t="s">
+      <c r="D98" s="193" t="s">
         <v>3096</v>
       </c>
     </row>
     <row r="99" spans="4:4">
-      <c r="D99" t="s">
+      <c r="D99" s="193" t="s">
         <v>3097</v>
       </c>
     </row>
     <row r="100" spans="4:4">
-      <c r="D100" t="s">
+      <c r="D100" s="193" t="s">
         <v>3098</v>
       </c>
     </row>
+    <row r="101" spans="4:4">
+      <c r="D101" s="193"/>
+    </row>
     <row r="102" spans="4:4">
-      <c r="D102" t="s">
+      <c r="D102" s="193" t="s">
         <v>3099</v>
       </c>
     </row>
     <row r="103" spans="4:4">
-      <c r="D103" t="s">
+      <c r="D103" s="193" t="s">
         <v>3100</v>
       </c>
     </row>
     <row r="104" spans="4:4">
-      <c r="D104" t="s">
+      <c r="D104" s="193" t="s">
         <v>3101</v>
       </c>
     </row>
+    <row r="105" spans="4:4">
+      <c r="D105" s="193"/>
+    </row>
     <row r="106" spans="4:4">
-      <c r="D106" t="s">
+      <c r="D106" s="193" t="s">
         <v>3102</v>
       </c>
     </row>
     <row r="107" spans="4:4">
-      <c r="D107" t="s">
+      <c r="D107" s="193" t="s">
         <v>3103</v>
       </c>
     </row>
     <row r="108" spans="4:4">
-      <c r="D108" t="s">
+      <c r="D108" s="193" t="s">
         <v>3104</v>
       </c>
     </row>
     <row r="109" spans="4:4">
-      <c r="D109" t="s">
+      <c r="D109" s="193" t="s">
         <v>3105</v>
       </c>
     </row>
     <row r="110" spans="4:4">
-      <c r="D110" t="s">
+      <c r="D110" s="193" t="s">
         <v>3106</v>
       </c>
     </row>
     <row r="111" spans="4:4">
-      <c r="D111" t="s">
+      <c r="D111" s="193" t="s">
         <v>3107</v>
       </c>
     </row>
     <row r="112" spans="4:4">
-      <c r="D112" t="s">
+      <c r="D112" s="193" t="s">
         <v>3108</v>
       </c>
     </row>
+    <row r="113" spans="4:4">
+      <c r="D113" s="193"/>
+    </row>
     <row r="114" spans="4:4">
-      <c r="D114" t="s">
+      <c r="D114" s="193" t="s">
         <v>3109</v>
       </c>
     </row>
     <row r="115" spans="4:4">
-      <c r="D115" t="s">
+      <c r="D115" s="193" t="s">
         <v>3110</v>
       </c>
     </row>
     <row r="116" spans="4:4">
-      <c r="D116" t="s">
+      <c r="D116" s="193" t="s">
         <v>3111</v>
       </c>
     </row>
     <row r="117" spans="4:4">
-      <c r="D117" t="s">
+      <c r="D117" s="193" t="s">
         <v>3112</v>
       </c>
     </row>
     <row r="118" spans="4:4">
-      <c r="D118" t="s">
+      <c r="D118" s="193" t="s">
         <v>3113</v>
       </c>
     </row>
+    <row r="119" spans="4:4">
+      <c r="D119" s="193"/>
+    </row>
     <row r="120" spans="4:4">
-      <c r="D120" t="s">
+      <c r="D120" s="193" t="s">
         <v>3114</v>
       </c>
     </row>
     <row r="121" spans="4:4">
-      <c r="D121" t="s">
+      <c r="D121" s="193" t="s">
         <v>3115</v>
       </c>
     </row>
     <row r="122" spans="4:4">
-      <c r="D122" t="s">
+      <c r="D122" s="193" t="s">
         <v>3116</v>
       </c>
     </row>
     <row r="123" spans="4:4">
-      <c r="D123" t="s">
+      <c r="D123" s="193" t="s">
         <v>3117</v>
       </c>
     </row>
+    <row r="124" spans="4:4">
+      <c r="D124" s="193"/>
+    </row>
     <row r="125" spans="4:4">
-      <c r="D125" t="s">
+      <c r="D125" s="193" t="s">
         <v>3118</v>
       </c>
     </row>
     <row r="126" spans="4:4">
-      <c r="D126" t="s">
+      <c r="D126" s="193" t="s">
         <v>3119</v>
       </c>
     </row>
     <row r="127" spans="4:4">
-      <c r="D127" t="s">
+      <c r="D127" s="193" t="s">
         <v>3120</v>
       </c>
     </row>
     <row r="128" spans="4:4">
-      <c r="D128" t="s">
+      <c r="D128" s="193" t="s">
         <v>3121</v>
       </c>
     </row>
     <row r="129" spans="4:4">
-      <c r="D129" t="s">
+      <c r="D129" s="193" t="s">
         <v>3122</v>
       </c>
     </row>
+    <row r="130" spans="4:4">
+      <c r="D130" s="193"/>
+    </row>
     <row r="131" spans="4:4">
-      <c r="D131" s="7" t="s">
+      <c r="D131" s="106" t="s">
         <v>3123</v>
       </c>
     </row>
     <row r="132" spans="4:4">
-      <c r="D132" s="20"/>
+      <c r="D132" s="107"/>
     </row>
     <row r="133" spans="4:4">
-      <c r="D133" s="22" t="s">
+      <c r="D133" s="113" t="s">
         <v>3127</v>
       </c>
     </row>
     <row r="134" spans="4:4">
-      <c r="D134" s="22" t="s">
+      <c r="D134" s="113" t="s">
         <v>3128</v>
       </c>
     </row>
     <row r="135" spans="4:4">
-      <c r="D135" s="25" t="s">
+      <c r="D135" s="108" t="s">
         <v>3124</v>
       </c>
     </row>
     <row r="136" spans="4:4">
-      <c r="D136" s="22" t="s">
+      <c r="D136" s="113" t="s">
         <v>3129</v>
       </c>
     </row>
     <row r="137" spans="4:4">
-      <c r="D137" s="22" t="s">
+      <c r="D137" s="113" t="s">
         <v>3130</v>
       </c>
     </row>
     <row r="138" spans="4:4">
-      <c r="D138" s="5"/>
+      <c r="D138" s="97"/>
     </row>
     <row r="139" spans="4:4">
-      <c r="D139" s="7" t="s">
+      <c r="D139" s="106" t="s">
         <v>3125</v>
       </c>
     </row>
     <row r="140" spans="4:4">
-      <c r="D140" s="5"/>
+      <c r="D140" s="97"/>
     </row>
     <row r="141" spans="4:4">
-      <c r="D141" s="8" t="s">
+      <c r="D141" s="95" t="s">
         <v>3126</v>
       </c>
     </row>
+    <row r="142" spans="4:4">
+      <c r="D142" s="193"/>
+    </row>
     <row r="143" spans="4:4">
-      <c r="D143" t="s">
+      <c r="D143" s="193" t="s">
         <v>3131</v>
       </c>
     </row>
     <row r="144" spans="4:4">
-      <c r="D144" t="s">
+      <c r="D144" s="193" t="s">
         <v>3132</v>
       </c>
     </row>
+    <row r="145" spans="4:4">
+      <c r="D145" s="193"/>
+    </row>
     <row r="146" spans="4:4">
-      <c r="D146" t="s">
+      <c r="D146" s="193" t="s">
         <v>3133</v>
       </c>
     </row>
     <row r="147" spans="4:4">
-      <c r="D147" t="s">
+      <c r="D147" s="193" t="s">
         <v>3134</v>
       </c>
     </row>
+    <row r="148" spans="4:4">
+      <c r="D148" s="193"/>
+    </row>
     <row r="149" spans="4:4">
-      <c r="D149" t="s">
+      <c r="D149" s="193" t="s">
         <v>3135</v>
       </c>
     </row>
+    <row r="150" spans="4:4">
+      <c r="D150" s="193"/>
+    </row>
     <row r="151" spans="4:4">
-      <c r="D151" s="7" t="s">
+      <c r="D151" s="106" t="s">
         <v>3136</v>
       </c>
     </row>
     <row r="152" spans="4:4">
-      <c r="D152" s="20"/>
+      <c r="D152" s="107"/>
     </row>
     <row r="153" spans="4:4">
-      <c r="D153" s="22" t="s">
+      <c r="D153" s="113" t="s">
         <v>3139</v>
       </c>
     </row>
     <row r="154" spans="4:4">
-      <c r="D154" s="22" t="s">
+      <c r="D154" s="113" t="s">
         <v>3140</v>
       </c>
     </row>
     <row r="155" spans="4:4">
-      <c r="D155" s="22" t="s">
+      <c r="D155" s="113" t="s">
         <v>3141</v>
       </c>
     </row>
     <row r="156" spans="4:4">
-      <c r="D156" s="22" t="s">
+      <c r="D156" s="113" t="s">
         <v>3142</v>
       </c>
     </row>
     <row r="157" spans="4:4">
-      <c r="D157" s="5"/>
+      <c r="D157" s="97"/>
     </row>
     <row r="158" spans="4:4">
-      <c r="D158" s="7" t="s">
+      <c r="D158" s="106" t="s">
         <v>3137</v>
       </c>
     </row>
     <row r="159" spans="4:4">
-      <c r="D159" s="20"/>
+      <c r="D159" s="107"/>
     </row>
     <row r="160" spans="4:4">
-      <c r="D160" s="22" t="s">
+      <c r="D160" s="113" t="s">
         <v>3143</v>
       </c>
     </row>
     <row r="161" spans="4:4">
-      <c r="D161" s="22" t="s">
+      <c r="D161" s="113" t="s">
         <v>3144</v>
       </c>
     </row>
     <row r="162" spans="4:4">
-      <c r="D162" s="184" t="s">
+      <c r="D162" s="221" t="s">
         <v>3145</v>
       </c>
     </row>
     <row r="163" spans="4:4">
-      <c r="D163" s="5"/>
+      <c r="D163" s="97"/>
     </row>
     <row r="164" spans="4:4">
-      <c r="D164" s="7" t="s">
+      <c r="D164" s="106" t="s">
         <v>3138</v>
       </c>
     </row>
+    <row r="165" spans="4:4">
+      <c r="D165" s="193"/>
+    </row>
     <row r="166" spans="4:4">
-      <c r="D166" t="s">
+      <c r="D166" s="193" t="s">
         <v>3146</v>
       </c>
     </row>
     <row r="167" spans="4:4">
-      <c r="D167" t="s">
+      <c r="D167" s="193" t="s">
         <v>3147</v>
       </c>
     </row>
     <row r="168" spans="4:4">
-      <c r="D168" t="s">
+      <c r="D168" s="193" t="s">
         <v>3148</v>
       </c>
     </row>
     <row r="169" spans="4:4">
-      <c r="D169" t="s">
+      <c r="D169" s="193" t="s">
         <v>3149</v>
       </c>
     </row>
     <row r="170" spans="4:4">
-      <c r="D170" t="s">
+      <c r="D170" s="193" t="s">
         <v>3150</v>
       </c>
     </row>
+    <row r="171" spans="4:4">
+      <c r="D171" s="193"/>
+    </row>
     <row r="172" spans="4:4">
-      <c r="D172" s="7" t="s">
+      <c r="D172" s="106" t="s">
         <v>3151</v>
       </c>
     </row>
     <row r="173" spans="4:4">
-      <c r="D173" s="8" t="s">
+      <c r="D173" s="95" t="s">
         <v>3152</v>
       </c>
     </row>
     <row r="174" spans="4:4">
-      <c r="D174" s="20"/>
+      <c r="D174" s="107"/>
     </row>
     <row r="175" spans="4:4">
-      <c r="D175" s="25" t="s">
+      <c r="D175" s="108" t="s">
         <v>3153</v>
       </c>
     </row>
     <row r="176" spans="4:4">
-      <c r="D176" s="21" t="s">
+      <c r="D176" s="109" t="s">
         <v>3154</v>
       </c>
     </row>
     <row r="177" spans="4:4">
-      <c r="D177" s="21" t="s">
+      <c r="D177" s="109" t="s">
         <v>3156</v>
       </c>
     </row>
     <row r="178" spans="4:4">
-      <c r="D178" s="21" t="s">
+      <c r="D178" s="109" t="s">
         <v>3157</v>
       </c>
     </row>
     <row r="179" spans="4:4">
-      <c r="D179" s="5"/>
+      <c r="D179" s="97"/>
     </row>
     <row r="180" spans="4:4">
-      <c r="D180" s="7" t="s">
+      <c r="D180" s="106" t="s">
         <v>3155</v>
+      </c>
+    </row>
+    <row r="182" spans="4:4" ht="30">
+      <c r="D182" s="156" t="s">
+        <v>3158</v>
+      </c>
+    </row>
+    <row r="184" spans="4:4" ht="28.5">
+      <c r="D184" s="95" t="s">
+        <v>3159</v>
+      </c>
+    </row>
+    <row r="186" spans="4:4">
+      <c r="D186" s="222" t="s">
+        <v>3160</v>
+      </c>
+    </row>
+    <row r="188" spans="4:4">
+      <c r="D188" s="222" t="s">
+        <v>3161</v>
+      </c>
+    </row>
+    <row r="190" spans="4:4" ht="28.5">
+      <c r="D190" s="89" t="s">
+        <v>3162</v>
+      </c>
+    </row>
+    <row r="192" spans="4:4" ht="42.75">
+      <c r="D192" s="8" t="s">
+        <v>3163</v>
+      </c>
+    </row>
+    <row r="193" spans="4:4">
+      <c r="D193" s="8" t="s">
+        <v>3164</v>
+      </c>
+    </row>
+    <row r="195" spans="4:4" ht="28.5">
+      <c r="D195" s="8" t="s">
+        <v>3186</v>
+      </c>
+    </row>
+    <row r="196" spans="4:4" ht="42.75">
+      <c r="D196" s="8" t="s">
+        <v>3165</v>
+      </c>
+    </row>
+    <row r="197" spans="4:4" ht="17.25">
+      <c r="D197" s="185" t="s">
+        <v>3166</v>
+      </c>
+    </row>
+    <row r="198" spans="4:4">
+      <c r="D198" s="7" t="s">
+        <v>3167</v>
+      </c>
+    </row>
+    <row r="199" spans="4:4">
+      <c r="D199" s="8" t="s">
+        <v>3168</v>
+      </c>
+    </row>
+    <row r="200" spans="4:4">
+      <c r="D200" s="8" t="s">
+        <v>3169</v>
+      </c>
+    </row>
+    <row r="201" spans="4:4">
+      <c r="D201" s="8" t="s">
+        <v>3170</v>
+      </c>
+    </row>
+    <row r="202" spans="4:4">
+      <c r="D202" s="16" t="s">
+        <v>3171</v>
+      </c>
+    </row>
+    <row r="203" spans="4:4">
+      <c r="D203" s="8" t="s">
+        <v>3172</v>
+      </c>
+    </row>
+    <row r="204" spans="4:4">
+      <c r="D204" s="7" t="s">
+        <v>3173</v>
+      </c>
+    </row>
+    <row r="205" spans="4:4" ht="28.5">
+      <c r="D205" s="8" t="s">
+        <v>3187</v>
+      </c>
+    </row>
+    <row r="206" spans="4:4">
+      <c r="D206" s="7" t="s">
+        <v>3174</v>
+      </c>
+    </row>
+    <row r="207" spans="4:4">
+      <c r="D207" s="20"/>
+    </row>
+    <row r="208" spans="4:4">
+      <c r="D208" s="25" t="s">
+        <v>3175</v>
+      </c>
+    </row>
+    <row r="209" spans="4:4">
+      <c r="D209" s="25" t="s">
+        <v>3176</v>
+      </c>
+    </row>
+    <row r="210" spans="4:4">
+      <c r="D210" s="25" t="s">
+        <v>3177</v>
+      </c>
+    </row>
+    <row r="211" spans="4:4">
+      <c r="D211" s="5"/>
+    </row>
+    <row r="212" spans="4:4">
+      <c r="D212" s="7" t="s">
+        <v>3178</v>
+      </c>
+    </row>
+    <row r="213" spans="4:4">
+      <c r="D213" s="8" t="s">
+        <v>3179</v>
+      </c>
+    </row>
+    <row r="214" spans="4:4">
+      <c r="D214" s="5"/>
+    </row>
+    <row r="215" spans="4:4" ht="28.5">
+      <c r="D215" s="7" t="s">
+        <v>3188</v>
+      </c>
+    </row>
+    <row r="216" spans="4:4">
+      <c r="D216" s="7" t="s">
+        <v>3189</v>
+      </c>
+    </row>
+    <row r="217" spans="4:4">
+      <c r="D217" s="20"/>
+    </row>
+    <row r="218" spans="4:4">
+      <c r="D218" s="21" t="s">
+        <v>3180</v>
+      </c>
+    </row>
+    <row r="219" spans="4:4">
+      <c r="D219" s="21" t="s">
+        <v>3181</v>
+      </c>
+    </row>
+    <row r="220" spans="4:4">
+      <c r="D220" s="21" t="s">
+        <v>3182</v>
+      </c>
+    </row>
+    <row r="221" spans="4:4">
+      <c r="D221" s="21" t="s">
+        <v>3183</v>
+      </c>
+    </row>
+    <row r="222" spans="4:4">
+      <c r="D222" s="21" t="s">
+        <v>3184</v>
+      </c>
+    </row>
+    <row r="223" spans="4:4">
+      <c r="D223" s="21" t="s">
+        <v>3185</v>
+      </c>
+    </row>
+    <row r="224" spans="4:4">
+      <c r="D224" s="5"/>
+    </row>
+    <row r="225" spans="4:4">
+      <c r="D225" s="7" t="s">
+        <v>3190</v>
+      </c>
+    </row>
+    <row r="226" spans="4:4">
+      <c r="D226" s="8" t="s">
+        <v>3038</v>
+      </c>
+    </row>
+    <row r="228" spans="4:4">
+      <c r="D228" s="193" t="s">
+        <v>3191</v>
+      </c>
+    </row>
+    <row r="230" spans="4:4">
+      <c r="D230" s="8" t="s">
+        <v>3192</v>
+      </c>
+    </row>
+    <row r="231" spans="4:4" ht="17.25">
+      <c r="D231" s="185" t="s">
+        <v>3193</v>
+      </c>
+    </row>
+    <row r="232" spans="4:4">
+      <c r="D232" s="7" t="s">
+        <v>3194</v>
+      </c>
+    </row>
+    <row r="233" spans="4:4">
+      <c r="D233" s="20"/>
+    </row>
+    <row r="234" spans="4:4">
+      <c r="D234" s="21" t="s">
+        <v>3195</v>
+      </c>
+    </row>
+    <row r="235" spans="4:4">
+      <c r="D235" s="21" t="s">
+        <v>3196</v>
+      </c>
+    </row>
+    <row r="236" spans="4:4">
+      <c r="D236" s="21" t="s">
+        <v>3197</v>
+      </c>
+    </row>
+    <row r="237" spans="4:4">
+      <c r="D237" s="5"/>
+    </row>
+    <row r="238" spans="4:4">
+      <c r="D238" s="7" t="s">
+        <v>3198</v>
+      </c>
+    </row>
+    <row r="239" spans="4:4">
+      <c r="D239" s="20"/>
+    </row>
+    <row r="240" spans="4:4" ht="30">
+      <c r="D240" s="25" t="s">
+        <v>3199</v>
+      </c>
+    </row>
+    <row r="241" spans="4:4">
+      <c r="D241" s="25" t="s">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="242" spans="4:4">
+      <c r="D242" s="5"/>
+    </row>
+    <row r="243" spans="4:4">
+      <c r="D243" s="7" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="245" spans="4:4" ht="30">
+      <c r="D245" s="6" t="s">
+        <v>3202</v>
+      </c>
+    </row>
+    <row r="246" spans="4:4">
+      <c r="D246" s="6"/>
+    </row>
+    <row r="247" spans="4:4">
+      <c r="D247" s="6" t="s">
+        <v>3203</v>
       </c>
     </row>
   </sheetData>
@@ -21792,7 +22596,176 @@
     <hyperlink ref="D80" r:id="rId11" display="vscode-file://vscode-app/c:/Users/tmsjd/AppData/Local/Programs/Microsoft VS Code/resources/app/out/vs/code/electron-browser/workbench/workbench.html"/>
     <hyperlink ref="D135" r:id="rId12" display="vscode-file://vscode-app/c:/Users/tmsjd/AppData/Local/Programs/Microsoft VS Code/resources/app/out/vs/code/electron-browser/workbench/workbench.html"/>
     <hyperlink ref="D175" r:id="rId13" display="vscode-file://vscode-app/c:/Users/tmsjd/AppData/Local/Programs/Microsoft VS Code/resources/app/out/vs/code/electron-browser/workbench/workbench.html"/>
+    <hyperlink ref="D202" r:id="rId14" display="vscode-file://vscode-app/c:/Users/tmsjd/AppData/Local/Programs/Microsoft VS Code/resources/app/out/vs/code/electron-browser/workbench/workbench.html"/>
+    <hyperlink ref="D208" r:id="rId15" display="vscode-file://vscode-app/c:/Users/tmsjd/AppData/Local/Programs/Microsoft VS Code/resources/app/out/vs/code/electron-browser/workbench/workbench.html"/>
+    <hyperlink ref="D209" r:id="rId16" display="vscode-file://vscode-app/c:/Users/tmsjd/AppData/Local/Programs/Microsoft VS Code/resources/app/out/vs/code/electron-browser/workbench/workbench.html"/>
+    <hyperlink ref="D210" r:id="rId17" display="vscode-file://vscode-app/c:/Users/tmsjd/AppData/Local/Programs/Microsoft VS Code/resources/app/out/vs/code/electron-browser/workbench/workbench.html"/>
+    <hyperlink ref="D240" r:id="rId18" display="vscode-file://vscode-app/c:/Users/tmsjd/AppData/Local/Programs/Microsoft VS Code/resources/app/out/vs/code/electron-browser/workbench/workbench.html"/>
+    <hyperlink ref="D241" r:id="rId19" display="vscode-file://vscode-app/c:/Users/tmsjd/AppData/Local/Programs/Microsoft VS Code/resources/app/out/vs/code/electron-browser/workbench/workbench.html"/>
   </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="D5:D36"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="4" max="4" width="91.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="4:4" ht="48">
+      <c r="D5" s="223" t="s">
+        <v>3204</v>
+      </c>
+    </row>
+    <row r="6" spans="4:4" ht="17.25">
+      <c r="D6" s="185" t="s">
+        <v>3205</v>
+      </c>
+    </row>
+    <row r="7" spans="4:4">
+      <c r="D7" s="8" t="s">
+        <v>3220</v>
+      </c>
+    </row>
+    <row r="8" spans="4:4">
+      <c r="D8" s="8" t="s">
+        <v>3221</v>
+      </c>
+    </row>
+    <row r="9" spans="4:4">
+      <c r="D9" s="8" t="s">
+        <v>3222</v>
+      </c>
+    </row>
+    <row r="10" spans="4:4">
+      <c r="D10" s="8" t="s">
+        <v>3223</v>
+      </c>
+    </row>
+    <row r="11" spans="4:4">
+      <c r="D11" s="8" t="s">
+        <v>3224</v>
+      </c>
+    </row>
+    <row r="12" spans="4:4">
+      <c r="D12" s="8" t="s">
+        <v>3225</v>
+      </c>
+    </row>
+    <row r="13" spans="4:4" ht="17.25">
+      <c r="D13" s="185" t="s">
+        <v>3206</v>
+      </c>
+    </row>
+    <row r="14" spans="4:4">
+      <c r="D14" s="7" t="s">
+        <v>3207</v>
+      </c>
+    </row>
+    <row r="15" spans="4:4" ht="28.5">
+      <c r="D15" s="8" t="s">
+        <v>3226</v>
+      </c>
+    </row>
+    <row r="16" spans="4:4" ht="17.25">
+      <c r="D16" s="185" t="s">
+        <v>3208</v>
+      </c>
+    </row>
+    <row r="17" spans="4:4">
+      <c r="D17" s="20"/>
+    </row>
+    <row r="18" spans="4:4">
+      <c r="D18" s="21" t="s">
+        <v>3209</v>
+      </c>
+    </row>
+    <row r="19" spans="4:4">
+      <c r="D19" s="21" t="s">
+        <v>3210</v>
+      </c>
+    </row>
+    <row r="20" spans="4:4">
+      <c r="D20" s="21" t="s">
+        <v>3211</v>
+      </c>
+    </row>
+    <row r="21" spans="4:4">
+      <c r="D21" s="21" t="s">
+        <v>3212</v>
+      </c>
+    </row>
+    <row r="22" spans="4:4">
+      <c r="D22" s="22" t="s">
+        <v>3227</v>
+      </c>
+    </row>
+    <row r="23" spans="4:4">
+      <c r="D23" s="5"/>
+    </row>
+    <row r="24" spans="4:4" ht="17.25">
+      <c r="D24" s="185" t="s">
+        <v>3213</v>
+      </c>
+    </row>
+    <row r="25" spans="4:4">
+      <c r="D25" s="20"/>
+    </row>
+    <row r="26" spans="4:4">
+      <c r="D26" s="21" t="s">
+        <v>3214</v>
+      </c>
+    </row>
+    <row r="27" spans="4:4">
+      <c r="D27" s="21" t="s">
+        <v>3215</v>
+      </c>
+    </row>
+    <row r="28" spans="4:4">
+      <c r="D28" s="21" t="s">
+        <v>3216</v>
+      </c>
+    </row>
+    <row r="29" spans="4:4">
+      <c r="D29" s="21" t="s">
+        <v>3217</v>
+      </c>
+    </row>
+    <row r="30" spans="4:4">
+      <c r="D30" s="21" t="s">
+        <v>3218</v>
+      </c>
+    </row>
+    <row r="31" spans="4:4">
+      <c r="D31" s="5"/>
+    </row>
+    <row r="32" spans="4:4">
+      <c r="D32" s="7" t="s">
+        <v>3219</v>
+      </c>
+    </row>
+    <row r="33" spans="4:4">
+      <c r="D33" s="20"/>
+    </row>
+    <row r="34" spans="4:4">
+      <c r="D34" s="22" t="s">
+        <v>3228</v>
+      </c>
+    </row>
+    <row r="35" spans="4:4">
+      <c r="D35" s="22" t="s">
+        <v>3229</v>
+      </c>
+    </row>
+    <row r="36" spans="4:4">
+      <c r="D36" s="22" t="s">
+        <v>3230</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -38954,7 +39927,7 @@
       </c>
     </row>
     <row r="691" spans="4:4">
-      <c r="D691" s="188" t="s">
+      <c r="D691" s="187" t="s">
         <v>2560</v>
       </c>
     </row>
@@ -39008,17 +39981,17 @@
       <c r="D702" s="82"/>
     </row>
     <row r="703" spans="4:4">
-      <c r="D703" s="189" t="s">
+      <c r="D703" s="188" t="s">
         <v>2563</v>
       </c>
     </row>
     <row r="704" spans="4:4">
-      <c r="D704" s="189" t="s">
+      <c r="D704" s="188" t="s">
         <v>2564</v>
       </c>
     </row>
     <row r="705" spans="4:4">
-      <c r="D705" s="189" t="s">
+      <c r="D705" s="188" t="s">
         <v>2565</v>
       </c>
     </row>
@@ -39218,12 +40191,12 @@
       </c>
     </row>
     <row r="750" spans="4:4">
-      <c r="D750" s="190" t="s">
+      <c r="D750" s="189" t="s">
         <v>2574</v>
       </c>
     </row>
     <row r="751" spans="4:4">
-      <c r="D751" s="190" t="s">
+      <c r="D751" s="189" t="s">
         <v>2575</v>
       </c>
     </row>
@@ -39256,7 +40229,7 @@
       </c>
     </row>
     <row r="760" spans="4:4" ht="17.25">
-      <c r="D760" s="191" t="s">
+      <c r="D760" s="190" t="s">
         <v>2600</v>
       </c>
     </row>
@@ -39475,7 +40448,7 @@
       <c r="D806" s="97"/>
     </row>
     <row r="807" spans="4:4" ht="17.25">
-      <c r="D807" s="191" t="s">
+      <c r="D807" s="190" t="s">
         <v>2621</v>
       </c>
     </row>
@@ -39559,141 +40532,141 @@
       </c>
     </row>
     <row r="828" spans="4:4" ht="17.25">
-      <c r="D828" s="194" t="s">
+      <c r="D828" s="195" t="s">
         <v>2650</v>
       </c>
     </row>
     <row r="829" spans="4:4">
-      <c r="D829" s="195" t="s">
+      <c r="D829" s="196" t="s">
         <v>2651</v>
       </c>
     </row>
     <row r="830" spans="4:4">
-      <c r="D830" s="196"/>
+      <c r="D830" s="197"/>
     </row>
     <row r="831" spans="4:4">
-      <c r="D831" s="196" t="s">
+      <c r="D831" s="197" t="s">
         <v>2159</v>
       </c>
     </row>
     <row r="832" spans="4:4">
-      <c r="D832" s="196" t="s">
+      <c r="D832" s="197" t="s">
         <v>2652</v>
       </c>
     </row>
     <row r="833" spans="4:4">
-      <c r="D833" s="196" t="s">
+      <c r="D833" s="197" t="s">
         <v>2653</v>
       </c>
     </row>
     <row r="834" spans="4:4">
-      <c r="D834" s="196" t="s">
+      <c r="D834" s="197" t="s">
         <v>2654</v>
       </c>
     </row>
     <row r="835" spans="4:4">
-      <c r="D835" s="196" t="s">
+      <c r="D835" s="197" t="s">
         <v>2325</v>
       </c>
     </row>
     <row r="836" spans="4:4">
-      <c r="D836" s="196" t="s">
+      <c r="D836" s="197" t="s">
         <v>2183</v>
       </c>
     </row>
     <row r="837" spans="4:4">
-      <c r="D837" s="196"/>
+      <c r="D837" s="197"/>
     </row>
     <row r="838" spans="4:4">
-      <c r="D838" s="197" t="s">
+      <c r="D838" s="198" t="s">
         <v>2655</v>
       </c>
     </row>
     <row r="839" spans="4:4">
-      <c r="D839" s="196"/>
+      <c r="D839" s="197"/>
     </row>
     <row r="840" spans="4:4">
-      <c r="D840" s="196" t="s">
+      <c r="D840" s="197" t="s">
         <v>2656</v>
       </c>
     </row>
     <row r="841" spans="4:4">
-      <c r="D841" s="196" t="s">
+      <c r="D841" s="197" t="s">
         <v>2657</v>
       </c>
     </row>
     <row r="842" spans="4:4">
-      <c r="D842" s="196" t="s">
+      <c r="D842" s="197" t="s">
         <v>2658</v>
       </c>
     </row>
     <row r="843" spans="4:4">
-      <c r="D843" s="196" t="s">
+      <c r="D843" s="197" t="s">
         <v>2121</v>
       </c>
     </row>
     <row r="844" spans="4:4">
-      <c r="D844" s="196" t="s">
+      <c r="D844" s="197" t="s">
         <v>2659</v>
       </c>
     </row>
     <row r="845" spans="4:4">
-      <c r="D845" s="196" t="s">
+      <c r="D845" s="197" t="s">
         <v>2660</v>
       </c>
     </row>
     <row r="846" spans="4:4">
-      <c r="D846" s="196" t="s">
+      <c r="D846" s="197" t="s">
         <v>2661</v>
       </c>
     </row>
     <row r="847" spans="4:4">
-      <c r="D847" s="196" t="s">
+      <c r="D847" s="197" t="s">
         <v>2662</v>
       </c>
     </row>
     <row r="848" spans="4:4">
-      <c r="D848" s="196" t="s">
+      <c r="D848" s="197" t="s">
         <v>2127</v>
       </c>
     </row>
     <row r="849" spans="4:4">
-      <c r="D849" s="196"/>
+      <c r="D849" s="197"/>
     </row>
     <row r="850" spans="4:4">
-      <c r="D850" s="195" t="s">
+      <c r="D850" s="196" t="s">
         <v>2663</v>
       </c>
     </row>
     <row r="851" spans="4:4">
-      <c r="D851" s="198"/>
+      <c r="D851" s="199"/>
     </row>
     <row r="852" spans="4:4">
-      <c r="D852" s="199" t="s">
+      <c r="D852" s="200" t="s">
         <v>2675</v>
       </c>
     </row>
     <row r="853" spans="4:4" ht="28.5">
-      <c r="D853" s="199" t="s">
+      <c r="D853" s="200" t="s">
         <v>2676</v>
       </c>
     </row>
     <row r="854" spans="4:4">
-      <c r="D854" s="200"/>
+      <c r="D854" s="201"/>
     </row>
     <row r="855" spans="4:4">
-      <c r="D855" s="201" t="s">
+      <c r="D855" s="202" t="s">
         <v>2677</v>
       </c>
     </row>
     <row r="856" spans="4:4">
-      <c r="D856" s="202"/>
+      <c r="D856" s="203"/>
     </row>
     <row r="857" spans="4:4">
-      <c r="D857" s="200"/>
+      <c r="D857" s="201"/>
     </row>
     <row r="858" spans="4:4">
-      <c r="D858" s="201" t="s">
+      <c r="D858" s="202" t="s">
         <v>2664</v>
       </c>
     </row>
@@ -39708,48 +40681,48 @@
       </c>
     </row>
     <row r="861" spans="4:4">
-      <c r="D861" s="198"/>
+      <c r="D861" s="199"/>
     </row>
     <row r="862" spans="4:4">
-      <c r="D862" s="203" t="s">
+      <c r="D862" s="204" t="s">
         <v>2667</v>
       </c>
     </row>
     <row r="863" spans="4:4">
-      <c r="D863" s="203" t="s">
+      <c r="D863" s="204" t="s">
         <v>2668</v>
       </c>
     </row>
     <row r="864" spans="4:4">
-      <c r="D864" s="203" t="s">
+      <c r="D864" s="204" t="s">
         <v>2669</v>
       </c>
     </row>
     <row r="865" spans="4:4">
-      <c r="D865" s="203" t="s">
+      <c r="D865" s="204" t="s">
         <v>2670</v>
       </c>
     </row>
     <row r="866" spans="4:4">
-      <c r="D866" s="203" t="s">
+      <c r="D866" s="204" t="s">
         <v>2671</v>
       </c>
     </row>
     <row r="867" spans="4:4">
-      <c r="D867" s="203" t="s">
+      <c r="D867" s="204" t="s">
         <v>2672</v>
       </c>
     </row>
     <row r="868" spans="4:4">
-      <c r="D868" s="203" t="s">
+      <c r="D868" s="204" t="s">
         <v>2673</v>
       </c>
     </row>
     <row r="869" spans="4:4">
-      <c r="D869" s="200"/>
+      <c r="D869" s="201"/>
     </row>
     <row r="870" spans="4:4">
-      <c r="D870" s="201" t="s">
+      <c r="D870" s="202" t="s">
         <v>2674</v>
       </c>
     </row>
@@ -39884,7 +40857,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="23.140625" customWidth="1"/>
-    <col min="4" max="4" width="37.7109375" style="192" customWidth="1"/>
+    <col min="4" max="4" width="37.7109375" style="191" customWidth="1"/>
     <col min="5" max="6" width="23" customWidth="1"/>
   </cols>
   <sheetData>
@@ -39892,639 +40865,639 @@
       <c r="B6" t="s">
         <v>2771</v>
       </c>
-      <c r="D6" s="207" t="s">
+      <c r="D6" s="208" t="s">
         <v>2678</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="16.5">
-      <c r="D7" s="208" t="s">
+      <c r="D7" s="209" t="s">
         <v>2679</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="49.5">
-      <c r="D8" s="208" t="s">
+      <c r="D8" s="209" t="s">
         <v>2680</v>
       </c>
     </row>
     <row r="9" spans="2:4">
-      <c r="D9" s="209"/>
+      <c r="D9" s="210"/>
     </row>
     <row r="10" spans="2:4" ht="99">
-      <c r="D10" s="210" t="s">
+      <c r="D10" s="211" t="s">
         <v>2681</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="99">
-      <c r="D11" s="210" t="s">
+      <c r="D11" s="211" t="s">
         <v>2682</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="115.5">
-      <c r="D12" s="210" t="s">
+      <c r="D12" s="211" t="s">
         <v>2683</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="99">
-      <c r="D13" s="208" t="s">
+      <c r="D13" s="209" t="s">
         <v>2684</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="42">
-      <c r="D16" s="207" t="s">
+      <c r="D16" s="208" t="s">
         <v>2685</v>
       </c>
     </row>
     <row r="17" spans="4:4" ht="33">
-      <c r="D17" s="208" t="s">
+      <c r="D17" s="209" t="s">
         <v>2686</v>
       </c>
     </row>
     <row r="18" spans="4:4" ht="33">
-      <c r="D18" s="208" t="s">
+      <c r="D18" s="209" t="s">
         <v>2687</v>
       </c>
     </row>
     <row r="19" spans="4:4">
-      <c r="D19" s="209"/>
+      <c r="D19" s="210"/>
     </row>
     <row r="20" spans="4:4" ht="49.5">
-      <c r="D20" s="210" t="s">
+      <c r="D20" s="211" t="s">
         <v>2772</v>
       </c>
     </row>
     <row r="21" spans="4:4" ht="82.5">
-      <c r="D21" s="210" t="s">
+      <c r="D21" s="211" t="s">
         <v>2688</v>
       </c>
     </row>
     <row r="22" spans="4:4" ht="30">
-      <c r="D22" s="211" t="s">
+      <c r="D22" s="212" t="s">
         <v>2689</v>
       </c>
     </row>
     <row r="23" spans="4:4" ht="33">
-      <c r="D23" s="208" t="s">
+      <c r="D23" s="209" t="s">
         <v>2690</v>
       </c>
     </row>
     <row r="24" spans="4:4">
-      <c r="D24" s="209"/>
+      <c r="D24" s="210"/>
     </row>
     <row r="25" spans="4:4" ht="16.5">
-      <c r="D25" s="210" t="s">
+      <c r="D25" s="211" t="s">
         <v>2691</v>
       </c>
     </row>
     <row r="26" spans="4:4" ht="49.5">
-      <c r="D26" s="210" t="s">
+      <c r="D26" s="211" t="s">
         <v>2692</v>
       </c>
     </row>
     <row r="27" spans="4:4" ht="33">
-      <c r="D27" s="210" t="s">
+      <c r="D27" s="211" t="s">
         <v>2693</v>
       </c>
     </row>
     <row r="28" spans="4:4" ht="82.5">
-      <c r="D28" s="210" t="s">
+      <c r="D28" s="211" t="s">
         <v>2694</v>
       </c>
     </row>
     <row r="29" spans="4:4" ht="16.5">
-      <c r="D29" s="210" t="s">
+      <c r="D29" s="211" t="s">
         <v>2695</v>
       </c>
     </row>
     <row r="30" spans="4:4" ht="45">
-      <c r="D30" s="211" t="s">
+      <c r="D30" s="212" t="s">
         <v>2696</v>
       </c>
     </row>
     <row r="31" spans="4:4" ht="26.25">
-      <c r="D31" s="212" t="s">
+      <c r="D31" s="213" t="s">
         <v>2697</v>
       </c>
     </row>
     <row r="32" spans="4:4" ht="66">
-      <c r="D32" s="208" t="s">
+      <c r="D32" s="209" t="s">
         <v>2698</v>
       </c>
     </row>
     <row r="35" spans="4:4" ht="42">
-      <c r="D35" s="207" t="s">
+      <c r="D35" s="208" t="s">
         <v>2699</v>
       </c>
     </row>
     <row r="36" spans="4:4">
-      <c r="D36" s="193" t="s">
+      <c r="D36" s="192" t="s">
         <v>2700</v>
       </c>
     </row>
     <row r="37" spans="4:4">
-      <c r="D37" s="193" t="s">
+      <c r="D37" s="192" t="s">
         <v>2701</v>
       </c>
     </row>
     <row r="38" spans="4:4">
-      <c r="D38" s="193" t="s">
+      <c r="D38" s="192" t="s">
         <v>2702</v>
       </c>
     </row>
     <row r="39" spans="4:4" ht="33">
-      <c r="D39" s="208" t="s">
+      <c r="D39" s="209" t="s">
         <v>2703</v>
       </c>
     </row>
     <row r="42" spans="4:4" ht="42">
-      <c r="D42" s="207" t="s">
+      <c r="D42" s="208" t="s">
         <v>2704</v>
       </c>
     </row>
     <row r="43" spans="4:4" ht="33">
-      <c r="D43" s="208" t="s">
+      <c r="D43" s="209" t="s">
         <v>2705</v>
       </c>
     </row>
     <row r="44" spans="4:4" ht="16.5">
-      <c r="D44" s="208" t="s">
+      <c r="D44" s="209" t="s">
         <v>2706</v>
       </c>
     </row>
     <row r="45" spans="4:4">
-      <c r="D45" s="192" t="s">
+      <c r="D45" s="191" t="s">
         <v>2707</v>
       </c>
     </row>
     <row r="46" spans="4:4">
-      <c r="D46" s="213" t="s">
+      <c r="D46" s="214" t="s">
         <v>2773</v>
       </c>
     </row>
     <row r="47" spans="4:4">
-      <c r="D47" s="213" t="s">
+      <c r="D47" s="214" t="s">
         <v>2774</v>
       </c>
     </row>
     <row r="48" spans="4:4" ht="30">
-      <c r="D48" s="213" t="s">
+      <c r="D48" s="214" t="s">
         <v>2775</v>
       </c>
     </row>
     <row r="49" spans="4:4">
-      <c r="D49" s="213" t="s">
+      <c r="D49" s="214" t="s">
         <v>2776</v>
       </c>
     </row>
     <row r="50" spans="4:4">
-      <c r="D50" s="213" t="s">
+      <c r="D50" s="214" t="s">
         <v>2777</v>
       </c>
     </row>
     <row r="51" spans="4:4">
-      <c r="D51" s="213" t="s">
+      <c r="D51" s="214" t="s">
         <v>2778</v>
       </c>
     </row>
     <row r="52" spans="4:4" ht="30">
-      <c r="D52" s="213" t="s">
+      <c r="D52" s="214" t="s">
         <v>2779</v>
       </c>
     </row>
     <row r="53" spans="4:4">
-      <c r="D53" s="213" t="s">
+      <c r="D53" s="214" t="s">
         <v>2780</v>
       </c>
     </row>
     <row r="54" spans="4:4">
-      <c r="D54" s="213" t="s">
+      <c r="D54" s="214" t="s">
         <v>2781</v>
       </c>
     </row>
     <row r="55" spans="4:4">
-      <c r="D55" s="213" t="s">
+      <c r="D55" s="214" t="s">
         <v>2782</v>
       </c>
     </row>
     <row r="56" spans="4:4">
-      <c r="D56" s="192" t="s">
+      <c r="D56" s="191" t="s">
         <v>2708</v>
       </c>
     </row>
     <row r="58" spans="4:4">
-      <c r="D58" s="192" t="s">
+      <c r="D58" s="191" t="s">
         <v>2709</v>
       </c>
     </row>
     <row r="59" spans="4:4" ht="45">
-      <c r="D59" s="213" t="s">
+      <c r="D59" s="214" t="s">
         <v>2783</v>
       </c>
     </row>
     <row r="60" spans="4:4" ht="30">
-      <c r="D60" s="213" t="s">
+      <c r="D60" s="214" t="s">
         <v>2784</v>
       </c>
     </row>
     <row r="61" spans="4:4" ht="30">
-      <c r="D61" s="213" t="s">
+      <c r="D61" s="214" t="s">
         <v>2785</v>
       </c>
     </row>
     <row r="62" spans="4:4" ht="30">
-      <c r="D62" s="213" t="s">
+      <c r="D62" s="214" t="s">
         <v>2786</v>
       </c>
     </row>
     <row r="63" spans="4:4" ht="45">
-      <c r="D63" s="213" t="s">
+      <c r="D63" s="214" t="s">
         <v>2787</v>
       </c>
     </row>
     <row r="64" spans="4:4" ht="30">
-      <c r="D64" s="192" t="s">
+      <c r="D64" s="191" t="s">
         <v>2710</v>
       </c>
     </row>
     <row r="66" spans="4:4">
-      <c r="D66" s="192" t="s">
+      <c r="D66" s="191" t="s">
         <v>2711</v>
       </c>
     </row>
     <row r="67" spans="4:4" ht="30">
-      <c r="D67" s="192" t="s">
+      <c r="D67" s="191" t="s">
         <v>2712</v>
       </c>
     </row>
     <row r="68" spans="4:4" ht="30">
-      <c r="D68" s="192" t="s">
+      <c r="D68" s="191" t="s">
         <v>2713</v>
       </c>
     </row>
     <row r="69" spans="4:4" ht="30">
-      <c r="D69" s="192" t="s">
+      <c r="D69" s="191" t="s">
         <v>2714</v>
       </c>
     </row>
     <row r="70" spans="4:4">
-      <c r="D70" s="192" t="s">
+      <c r="D70" s="191" t="s">
         <v>2715</v>
       </c>
     </row>
     <row r="71" spans="4:4">
-      <c r="D71" s="192" t="s">
+      <c r="D71" s="191" t="s">
         <v>2716</v>
       </c>
     </row>
     <row r="72" spans="4:4" ht="30">
-      <c r="D72" s="192" t="s">
+      <c r="D72" s="191" t="s">
         <v>2717</v>
       </c>
     </row>
     <row r="74" spans="4:4" ht="16.5">
-      <c r="D74" s="208" t="s">
+      <c r="D74" s="209" t="s">
         <v>2718</v>
       </c>
     </row>
     <row r="75" spans="4:4" ht="66">
-      <c r="D75" s="208" t="s">
+      <c r="D75" s="209" t="s">
         <v>2719</v>
       </c>
     </row>
     <row r="76" spans="4:4" ht="16.5">
-      <c r="D76" s="208"/>
+      <c r="D76" s="209"/>
     </row>
     <row r="77" spans="4:4" ht="33">
-      <c r="D77" s="208" t="s">
+      <c r="D77" s="209" t="s">
         <v>2720</v>
       </c>
     </row>
     <row r="78" spans="4:4" ht="16.5">
-      <c r="D78" s="208" t="s">
+      <c r="D78" s="209" t="s">
         <v>2706</v>
       </c>
     </row>
     <row r="79" spans="4:4" ht="16.5">
-      <c r="D79" s="208" t="s">
+      <c r="D79" s="209" t="s">
         <v>2721</v>
       </c>
     </row>
     <row r="80" spans="4:4" ht="16.5">
-      <c r="D80" s="213" t="s">
+      <c r="D80" s="214" t="s">
         <v>2788</v>
       </c>
     </row>
     <row r="81" spans="4:4" ht="16.5">
-      <c r="D81" s="213" t="s">
+      <c r="D81" s="214" t="s">
         <v>2789</v>
       </c>
     </row>
     <row r="82" spans="4:4" ht="16.5">
-      <c r="D82" s="213" t="s">
+      <c r="D82" s="214" t="s">
         <v>2790</v>
       </c>
     </row>
     <row r="83" spans="4:4" ht="16.5">
-      <c r="D83" s="213" t="s">
+      <c r="D83" s="214" t="s">
         <v>2791</v>
       </c>
     </row>
     <row r="84" spans="4:4" ht="16.5">
-      <c r="D84" s="213" t="s">
+      <c r="D84" s="214" t="s">
         <v>2792</v>
       </c>
     </row>
     <row r="85" spans="4:4" ht="16.5">
-      <c r="D85" s="213" t="s">
+      <c r="D85" s="214" t="s">
         <v>2793</v>
       </c>
     </row>
     <row r="86" spans="4:4" ht="16.5">
-      <c r="D86" s="213" t="s">
+      <c r="D86" s="214" t="s">
         <v>2794</v>
       </c>
     </row>
     <row r="87" spans="4:4" ht="16.5">
-      <c r="D87" s="213" t="s">
+      <c r="D87" s="214" t="s">
         <v>2795</v>
       </c>
     </row>
     <row r="88" spans="4:4" ht="16.5">
-      <c r="D88" s="213" t="s">
+      <c r="D88" s="214" t="s">
         <v>2796</v>
       </c>
     </row>
     <row r="89" spans="4:4" ht="33">
-      <c r="D89" s="213" t="s">
+      <c r="D89" s="214" t="s">
         <v>2797</v>
       </c>
     </row>
     <row r="90" spans="4:4" ht="16.5">
-      <c r="D90" s="208"/>
+      <c r="D90" s="209"/>
     </row>
     <row r="91" spans="4:4" ht="16.5">
-      <c r="D91" s="208" t="s">
+      <c r="D91" s="209" t="s">
         <v>2722</v>
       </c>
     </row>
     <row r="92" spans="4:4" ht="16.5">
-      <c r="D92" s="213" t="s">
+      <c r="D92" s="214" t="s">
         <v>2798</v>
       </c>
     </row>
     <row r="93" spans="4:4" ht="33">
-      <c r="D93" s="213" t="s">
+      <c r="D93" s="214" t="s">
         <v>2799</v>
       </c>
     </row>
     <row r="94" spans="4:4" ht="33">
-      <c r="D94" s="213" t="s">
+      <c r="D94" s="214" t="s">
         <v>2800</v>
       </c>
     </row>
     <row r="95" spans="4:4" ht="33">
-      <c r="D95" s="213" t="s">
+      <c r="D95" s="214" t="s">
         <v>2801</v>
       </c>
     </row>
     <row r="96" spans="4:4" ht="33">
-      <c r="D96" s="213" t="s">
+      <c r="D96" s="214" t="s">
         <v>2802</v>
       </c>
     </row>
     <row r="97" spans="2:6" ht="33">
-      <c r="D97" s="213" t="s">
+      <c r="D97" s="214" t="s">
         <v>2803</v>
       </c>
     </row>
     <row r="98" spans="2:6" ht="33">
-      <c r="D98" s="213" t="s">
+      <c r="D98" s="214" t="s">
         <v>2804</v>
       </c>
     </row>
     <row r="99" spans="2:6" ht="16.5">
-      <c r="D99" s="208"/>
+      <c r="D99" s="209"/>
     </row>
     <row r="100" spans="2:6" ht="16.5">
-      <c r="D100" s="208" t="s">
+      <c r="D100" s="209" t="s">
         <v>2723</v>
       </c>
     </row>
     <row r="101" spans="2:6" ht="33">
-      <c r="D101" s="208" t="s">
+      <c r="D101" s="209" t="s">
         <v>2724</v>
       </c>
     </row>
     <row r="102" spans="2:6" ht="16.5">
-      <c r="D102" s="208" t="s">
+      <c r="D102" s="209" t="s">
         <v>2725</v>
       </c>
     </row>
     <row r="103" spans="2:6" ht="16.5">
-      <c r="D103" s="208" t="s">
+      <c r="D103" s="209" t="s">
         <v>2726</v>
       </c>
     </row>
     <row r="104" spans="2:6" ht="33">
-      <c r="D104" s="208" t="s">
+      <c r="D104" s="209" t="s">
         <v>2727</v>
       </c>
     </row>
     <row r="105" spans="2:6" ht="33">
-      <c r="D105" s="208" t="s">
+      <c r="D105" s="209" t="s">
         <v>2728</v>
       </c>
     </row>
     <row r="106" spans="2:6" ht="33">
-      <c r="D106" s="208" t="s">
+      <c r="D106" s="209" t="s">
         <v>2729</v>
       </c>
     </row>
     <row r="107" spans="2:6" ht="16.5">
-      <c r="D107" s="208"/>
+      <c r="D107" s="209"/>
     </row>
     <row r="108" spans="2:6" ht="16.5">
-      <c r="D108" s="208" t="s">
+      <c r="D108" s="209" t="s">
         <v>2718</v>
       </c>
     </row>
     <row r="109" spans="2:6" ht="66">
-      <c r="D109" s="208" t="s">
+      <c r="D109" s="209" t="s">
         <v>2730</v>
       </c>
     </row>
     <row r="110" spans="2:6" ht="16.5">
-      <c r="D110" s="208"/>
+      <c r="D110" s="209"/>
     </row>
     <row r="111" spans="2:6" ht="21.75" thickBot="1">
-      <c r="B111" s="205"/>
-      <c r="D111" s="207" t="s">
+      <c r="B111" s="206"/>
+      <c r="D111" s="208" t="s">
         <v>2731</v>
       </c>
     </row>
-    <row r="112" spans="2:6" s="205" customFormat="1" ht="33.75" thickBot="1">
-      <c r="D112" s="214" t="s">
+    <row r="112" spans="2:6" s="206" customFormat="1" ht="33.75" thickBot="1">
+      <c r="D112" s="215" t="s">
         <v>2732</v>
       </c>
-      <c r="E112" s="204" t="s">
+      <c r="E112" s="205" t="s">
         <v>2733</v>
       </c>
-      <c r="F112" s="204" t="s">
+      <c r="F112" s="205" t="s">
         <v>2734</v>
       </c>
     </row>
-    <row r="113" spans="2:6" s="205" customFormat="1" ht="33.75" thickBot="1">
-      <c r="D113" s="215" t="s">
+    <row r="113" spans="2:6" s="206" customFormat="1" ht="33.75" thickBot="1">
+      <c r="D113" s="216" t="s">
         <v>2735</v>
       </c>
-      <c r="E113" s="206" t="s">
+      <c r="E113" s="207" t="s">
         <v>2736</v>
       </c>
-      <c r="F113" s="206" t="s">
+      <c r="F113" s="207" t="s">
         <v>2737</v>
       </c>
     </row>
-    <row r="114" spans="2:6" s="205" customFormat="1" ht="33.75" thickBot="1">
-      <c r="D114" s="215" t="s">
+    <row r="114" spans="2:6" s="206" customFormat="1" ht="33.75" thickBot="1">
+      <c r="D114" s="216" t="s">
         <v>2738</v>
       </c>
-      <c r="E114" s="206" t="s">
+      <c r="E114" s="207" t="s">
         <v>2739</v>
       </c>
-      <c r="F114" s="206" t="s">
+      <c r="F114" s="207" t="s">
         <v>2740</v>
       </c>
     </row>
-    <row r="115" spans="2:6" s="205" customFormat="1" ht="50.25" thickBot="1">
-      <c r="D115" s="215" t="s">
+    <row r="115" spans="2:6" s="206" customFormat="1" ht="50.25" thickBot="1">
+      <c r="D115" s="216" t="s">
         <v>2741</v>
       </c>
-      <c r="E115" s="206" t="s">
+      <c r="E115" s="207" t="s">
         <v>2742</v>
       </c>
-      <c r="F115" s="206" t="s">
+      <c r="F115" s="207" t="s">
         <v>2743</v>
       </c>
     </row>
-    <row r="116" spans="2:6" s="205" customFormat="1" ht="50.25" thickBot="1">
-      <c r="D116" s="215" t="s">
+    <row r="116" spans="2:6" s="206" customFormat="1" ht="50.25" thickBot="1">
+      <c r="D116" s="216" t="s">
         <v>2744</v>
       </c>
-      <c r="E116" s="206" t="s">
+      <c r="E116" s="207" t="s">
         <v>2745</v>
       </c>
-      <c r="F116" s="206" t="s">
+      <c r="F116" s="207" t="s">
         <v>2746</v>
       </c>
     </row>
-    <row r="117" spans="2:6" s="205" customFormat="1" ht="33.75" thickBot="1">
-      <c r="D117" s="215" t="s">
+    <row r="117" spans="2:6" s="206" customFormat="1" ht="33.75" thickBot="1">
+      <c r="D117" s="216" t="s">
         <v>2747</v>
       </c>
-      <c r="E117" s="206" t="s">
+      <c r="E117" s="207" t="s">
         <v>2748</v>
       </c>
-      <c r="F117" s="206" t="s">
+      <c r="F117" s="207" t="s">
         <v>2749</v>
       </c>
     </row>
-    <row r="118" spans="2:6" s="205" customFormat="1" ht="33.75" thickBot="1">
-      <c r="D118" s="215" t="s">
+    <row r="118" spans="2:6" s="206" customFormat="1" ht="33.75" thickBot="1">
+      <c r="D118" s="216" t="s">
         <v>2750</v>
       </c>
-      <c r="E118" s="206" t="s">
+      <c r="E118" s="207" t="s">
         <v>2751</v>
       </c>
-      <c r="F118" s="206" t="s">
+      <c r="F118" s="207" t="s">
         <v>2752</v>
       </c>
     </row>
-    <row r="119" spans="2:6" s="205" customFormat="1" ht="50.25" thickBot="1">
-      <c r="D119" s="215" t="s">
+    <row r="119" spans="2:6" s="206" customFormat="1" ht="50.25" thickBot="1">
+      <c r="D119" s="216" t="s">
         <v>2753</v>
       </c>
-      <c r="E119" s="206" t="s">
+      <c r="E119" s="207" t="s">
         <v>2754</v>
       </c>
-      <c r="F119" s="206" t="s">
+      <c r="F119" s="207" t="s">
         <v>2755</v>
       </c>
     </row>
-    <row r="120" spans="2:6" s="205" customFormat="1" ht="33.75" thickBot="1">
-      <c r="D120" s="215" t="s">
+    <row r="120" spans="2:6" s="206" customFormat="1" ht="33.75" thickBot="1">
+      <c r="D120" s="216" t="s">
         <v>2756</v>
       </c>
-      <c r="E120" s="206" t="s">
+      <c r="E120" s="207" t="s">
         <v>2757</v>
       </c>
-      <c r="F120" s="206" t="s">
+      <c r="F120" s="207" t="s">
         <v>2749</v>
       </c>
     </row>
-    <row r="121" spans="2:6" s="205" customFormat="1" ht="33.75" thickBot="1">
+    <row r="121" spans="2:6" s="206" customFormat="1" ht="33.75" thickBot="1">
       <c r="B121"/>
-      <c r="D121" s="215" t="s">
+      <c r="D121" s="216" t="s">
         <v>2758</v>
       </c>
-      <c r="E121" s="206" t="s">
+      <c r="E121" s="207" t="s">
         <v>2759</v>
       </c>
-      <c r="F121" s="206" t="s">
+      <c r="F121" s="207" t="s">
         <v>2760</v>
       </c>
     </row>
     <row r="124" spans="2:6" ht="42">
-      <c r="D124" s="207" t="s">
+      <c r="D124" s="208" t="s">
         <v>2761</v>
       </c>
     </row>
     <row r="125" spans="2:6" ht="82.5">
-      <c r="D125" s="208" t="s">
+      <c r="D125" s="209" t="s">
         <v>2762</v>
       </c>
     </row>
     <row r="126" spans="2:6">
-      <c r="D126" s="209"/>
+      <c r="D126" s="210"/>
     </row>
     <row r="127" spans="2:6" ht="30">
-      <c r="D127" s="211" t="s">
+      <c r="D127" s="212" t="s">
         <v>2763</v>
       </c>
     </row>
     <row r="128" spans="2:6" ht="30">
-      <c r="D128" s="211" t="s">
+      <c r="D128" s="212" t="s">
         <v>2764</v>
       </c>
     </row>
     <row r="129" spans="4:4" ht="49.5">
-      <c r="D129" s="210" t="s">
+      <c r="D129" s="211" t="s">
         <v>2765</v>
       </c>
     </row>
     <row r="130" spans="4:4" ht="16.5">
-      <c r="D130" s="208" t="s">
+      <c r="D130" s="209" t="s">
         <v>2766</v>
       </c>
     </row>
     <row r="131" spans="4:4">
-      <c r="D131" s="209"/>
+      <c r="D131" s="210"/>
     </row>
     <row r="132" spans="4:4" ht="49.5">
-      <c r="D132" s="210" t="s">
+      <c r="D132" s="211" t="s">
         <v>2767</v>
       </c>
     </row>
     <row r="133" spans="4:4" ht="49.5">
-      <c r="D133" s="210" t="s">
+      <c r="D133" s="211" t="s">
         <v>2768</v>
       </c>
     </row>
     <row r="134" spans="4:4" ht="115.5">
-      <c r="D134" s="208" t="s">
+      <c r="D134" s="209" t="s">
         <v>2769</v>
       </c>
     </row>
     <row r="135" spans="4:4" ht="49.5">
-      <c r="D135" s="208" t="s">
+      <c r="D135" s="209" t="s">
         <v>2770</v>
       </c>
     </row>

</xml_diff>